<commit_message>
Agrega hash de integridad y datos de congelacion a la matriz
</commit_message>
<xml_diff>
--- a/Registro_Experimento_WaterSOS.xlsx
+++ b/Registro_Experimento_WaterSOS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ISC_A\OneDrive\Documentos\Escuela\Investigacion\Titulaciones de Investigacion y Tesis\Nicazio Tesis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\RepWatOriginal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D7FAFC-BEF5-497D-857E-5AE360A11071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341B57EA-5576-4C9E-9D16-D8E6071A60D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="267">
   <si>
     <t>Registro de experimentación — WaterSOS / REPFUAGUA</t>
   </si>
@@ -826,6 +826,27 @@
   </si>
   <si>
     <t>Se confirma CWE-798 (Use of Hard-coded Credentials) en conexion.php: las credenciales de conexión a MySQL (usuario root, contraseña vacía) están escritas en texto plano directamente en el código fuente, en vez de estar en variables de entorno o un archivo de configuración externo al control de versiones. Se validó en phpMyAdmin que el servidor opera activamente con la sesión root@localhost sin SSL, confirmando que esas credenciales fijas son las reales y otorgan acceso administrativo total al motor de base de datos desde cualquier copia del código fuente. Como hallazgo complementario del mismo principio, se detectó que la app Android fija la dirección IP del servidor directamente en el código (EnviarDatos.java, líneas 171-172, literal 192.168.1.66) en lugar de externalizarla a un archivo de configuración, además de una entrada inconsistente de IP/puerto en strings.xml (192.168.1.70:8080) que no se utiliza en las llamadas reales al servicio.</t>
+  </si>
+  <si>
+    <t>https://github.com/AlfonsoRE/watersos-repfuagua-linea-base</t>
+  </si>
+  <si>
+    <t>linea-base-v1.0</t>
+  </si>
+  <si>
+    <t>e065fbc7075b9efe8104ae4718cecee368b5764d</t>
+  </si>
+  <si>
+    <t>Repositorio línea base:</t>
+  </si>
+  <si>
+    <t>Tag de congelación:</t>
+  </si>
+  <si>
+    <t>Hash de integridad (commit):</t>
+  </si>
+  <si>
+    <t>Fecha de congelación:</t>
   </si>
 </sst>
 </file>
@@ -836,7 +857,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -888,6 +909,13 @@
       <color rgb="FFA6A6A6"/>
       <name val="Arial"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -961,7 +989,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1074,6 +1102,16 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1848,7 +1886,7 @@
     <tabColor rgb="FF1F4E78"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -1879,307 +1917,226 @@
       <c r="J1" s="32"/>
       <c r="K1" s="32"/>
     </row>
-    <row r="3" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="42" t="s">
+        <v>263</v>
+      </c>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="40" t="s">
+        <v>260</v>
+      </c>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="42" t="s">
+        <v>264</v>
+      </c>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="40" t="s">
+        <v>261</v>
+      </c>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
+      <c r="K4" s="40"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="42" t="s">
+        <v>265</v>
+      </c>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="40" t="s">
+        <v>262</v>
+      </c>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
+      <c r="K5" s="40"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="42" t="s">
+        <v>266</v>
+      </c>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="41">
+        <v>46316</v>
+      </c>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="40"/>
+      <c r="K6" s="40"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="43"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+    </row>
+    <row r="8" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B8" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D8" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F8" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G8" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H8" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I8" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J8" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K8" s="7" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="51" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+    <row r="9" spans="1:11" ht="51" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B9" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C9" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D9" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>100</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="H4" s="10">
-        <v>46304</v>
-      </c>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="11" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="102" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="H5" s="10">
-        <v>46304</v>
-      </c>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="11" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="H6" s="10">
-        <v>46304</v>
-      </c>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="11" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="H7" s="10">
-        <v>46311</v>
-      </c>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="11" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="102" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>178</v>
-      </c>
-      <c r="H8" s="10">
-        <v>46311</v>
-      </c>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="11" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>117</v>
       </c>
       <c r="G9" s="9" t="s">
         <v>237</v>
       </c>
       <c r="H9" s="10">
-        <v>46311</v>
+        <v>46304</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
       <c r="K9" s="11" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="114.75" x14ac:dyDescent="0.25">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="102" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>237</v>
       </c>
       <c r="H10" s="10">
-        <v>46311</v>
+        <v>46304</v>
       </c>
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
       <c r="K10" s="11" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="102" x14ac:dyDescent="0.25">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="G11" s="9" t="s">
         <v>237</v>
       </c>
       <c r="H11" s="10">
-        <v>46311</v>
+        <v>46304</v>
       </c>
       <c r="I11" s="9"/>
       <c r="J11" s="9"/>
       <c r="K11" s="11" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="127.5" x14ac:dyDescent="0.25">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>237</v>
@@ -2190,30 +2147,30 @@
       <c r="I12" s="9"/>
       <c r="J12" s="9"/>
       <c r="K12" s="11" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="191.25" x14ac:dyDescent="0.25">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="102" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>116</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>237</v>
+        <v>178</v>
       </c>
       <c r="H13" s="10">
         <v>46311</v>
@@ -2221,154 +2178,317 @@
       <c r="I13" s="9"/>
       <c r="J13" s="9"/>
       <c r="K13" s="11" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="255" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>139</v>
+        <v>116</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>237</v>
       </c>
       <c r="H14" s="10">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="I14" s="9"/>
       <c r="J14" s="9"/>
       <c r="K14" s="11" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="204" x14ac:dyDescent="0.25">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>141</v>
+        <v>120</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>139</v>
+        <v>116</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>237</v>
       </c>
       <c r="H15" s="10">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="I15" s="9"/>
       <c r="J15" s="9"/>
       <c r="K15" s="11" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="153" x14ac:dyDescent="0.25">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="102" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>50</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>139</v>
+        <v>116</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>237</v>
       </c>
       <c r="H16" s="10">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="I16" s="9"/>
       <c r="J16" s="9"/>
       <c r="K16" s="11" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="114.75" x14ac:dyDescent="0.25">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>139</v>
+        <v>116</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>237</v>
       </c>
       <c r="H17" s="10">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="I17" s="9"/>
       <c r="J17" s="9"/>
       <c r="K17" s="11" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="191.25" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="H18" s="10">
+        <v>46311</v>
+      </c>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="11" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="255" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="H19" s="10">
+        <v>46316</v>
+      </c>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="11" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="204" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="H20" s="10">
+        <v>46316</v>
+      </c>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="11" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="153" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="H21" s="10">
+        <v>46316</v>
+      </c>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="11" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="H22" s="10">
+        <v>46316</v>
+      </c>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="11" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="36" t="s">
+    <row r="24" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="36" t="s">
         <v>151</v>
       </c>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="36"/>
-      <c r="K19" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="36"/>
+      <c r="J24" s="36"/>
+      <c r="K24" s="36"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="10">
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="B19:K19"/>
+    <mergeCell ref="B24:K24"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:K3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E4:K4"/>
+    <mergeCell ref="E5:K5"/>
+    <mergeCell ref="E6:K6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="G4:G17" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="G9:G22" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Sí,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6795,7 +6915,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0300-000002000000}">
           <x14:formula1>
-            <xm:f>Matriz_Casos_Prueba!$A$4:$A$17</xm:f>
+            <xm:f>Matriz_Casos_Prueba!$A$9:$A$22</xm:f>
           </x14:formula1>
           <x14:formula2>
             <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Actualiza matriz de registro del experimento
</commit_message>
<xml_diff>
--- a/Registro_Experimento_WaterSOS.xlsx
+++ b/Registro_Experimento_WaterSOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\RepWatOriginal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341B57EA-5576-4C9E-9D16-D8E6071A60D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E5A9F8-742C-4B8A-853C-A9F84D389965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -834,9 +834,6 @@
     <t>linea-base-v1.0</t>
   </si>
   <si>
-    <t>e065fbc7075b9efe8104ae4718cecee368b5764d</t>
-  </si>
-  <si>
     <t>Repositorio línea base:</t>
   </si>
   <si>
@@ -847,6 +844,9 @@
   </si>
   <si>
     <t>Fecha de congelación:</t>
+  </si>
+  <si>
+    <t>e605fbc7075b9efe8104ae4718cecee368b5764d</t>
   </si>
 </sst>
 </file>
@@ -1079,6 +1079,7 @@
     <xf numFmtId="165" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1093,6 +1094,15 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1102,16 +1112,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1389,41 +1389,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
+      <c r="A1" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
     </row>
     <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="34"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="34"/>
+      <c r="C4" s="35"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="31"/>
+      <c r="C6" s="32"/>
     </row>
     <row r="7" spans="1:3" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="35"/>
+      <c r="C7" s="36"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="31"/>
+      <c r="C9" s="32"/>
     </row>
     <row r="10" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
@@ -1482,10 +1482,10 @@
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="31"/>
+      <c r="C18" s="32"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
@@ -1512,10 +1512,10 @@
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="31"/>
+      <c r="C23" s="32"/>
     </row>
     <row r="24" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="6" t="s">
@@ -1608,16 +1608,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -1854,15 +1854,15 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="37" t="s">
         <v>84</v>
       </c>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="36"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1903,93 +1903,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="38" t="s">
+        <v>262</v>
+      </c>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="39" t="s">
+        <v>260</v>
+      </c>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="38" t="s">
         <v>263</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="40" t="s">
-        <v>260</v>
-      </c>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="39" t="s">
+        <v>261</v>
+      </c>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="38" t="s">
         <v>264</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="40" t="s">
-        <v>261</v>
-      </c>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
-      <c r="I4" s="40"/>
-      <c r="J4" s="40"/>
-      <c r="K4" s="40"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="39"/>
+      <c r="I5" s="39"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="39"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="38" t="s">
         <v>265</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="40" t="s">
-        <v>262</v>
-      </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="40"/>
-      <c r="I5" s="40"/>
-      <c r="J5" s="40"/>
-      <c r="K5" s="40"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="42" t="s">
-        <v>266</v>
-      </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="42"/>
-      <c r="E6" s="41">
+      <c r="B6" s="38"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="40">
         <v>46316</v>
       </c>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="40"/>
-      <c r="K6" s="40"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
+      <c r="A7" s="31"/>
+      <c r="B7" s="31"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
     </row>
     <row r="8" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
@@ -2461,18 +2461,18 @@
       </c>
     </row>
     <row r="24" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="37" t="s">
         <v>151</v>
       </c>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="36"/>
-      <c r="K24" s="36"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="37"/>
+      <c r="K24" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2526,25 +2526,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="33"/>
     </row>
     <row r="3" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -6956,17 +6956,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>180</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -9938,17 +9938,17 @@
       </c>
     </row>
     <row r="89" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="36" t="s">
+      <c r="A89" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="B89" s="36"/>
-      <c r="C89" s="36"/>
-      <c r="D89" s="36"/>
-      <c r="E89" s="36"/>
-      <c r="F89" s="36"/>
-      <c r="G89" s="36"/>
-      <c r="H89" s="36"/>
-      <c r="I89" s="36"/>
+      <c r="B89" s="37"/>
+      <c r="C89" s="37"/>
+      <c r="D89" s="37"/>
+      <c r="E89" s="37"/>
+      <c r="F89" s="37"/>
+      <c r="G89" s="37"/>
+      <c r="H89" s="37"/>
+      <c r="I89" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -9977,15 +9977,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -10049,15 +10049,15 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="37" t="s">
         <v>200</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -10085,12 +10085,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>201</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
     </row>
     <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -10250,12 +10250,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
@@ -10398,21 +10398,21 @@
       <c r="D12" s="11"/>
     </row>
     <row r="14" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
     </row>
     <row r="15" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
         <v>233</v>
       </c>
-      <c r="B15" s="37">
+      <c r="B15" s="41">
         <v>0.1</v>
       </c>
-      <c r="C15" s="37"/>
+      <c r="C15" s="41"/>
       <c r="D15" s="11" t="s">
         <v>234</v>
       </c>
@@ -10421,22 +10421,22 @@
       <c r="A16" s="26" t="s">
         <v>235</v>
       </c>
-      <c r="B16" s="38">
+      <c r="B16" s="42">
         <f>IFERROR(ABS(B4-C4),"")</f>
         <v>2.3809523809523808E-2</v>
       </c>
-      <c r="C16" s="38"/>
+      <c r="C16" s="42"/>
       <c r="D16" s="11"/>
     </row>
     <row r="17" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
         <v>236</v>
       </c>
-      <c r="B17" s="39" t="str">
+      <c r="B17" s="43" t="str">
         <f>IFERROR(IF(B16&lt;=B15,"Sí, dentro del margen","No, fuera del margen"),"")</f>
         <v>Sí, dentro del margen</v>
       </c>
-      <c r="C17" s="39"/>
+      <c r="C17" s="43"/>
       <c r="D17" s="11"/>
     </row>
   </sheetData>

</xml_diff>